<commit_message>
feat: implement enterprise data security, integration services, and validation audit artifacts
</commit_message>
<xml_diff>
--- a/MODULE_1_EXCEPTION_LEDGER.xlsx
+++ b/MODULE_1_EXCEPTION_LEDGER.xlsx
@@ -32,9 +32,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-    <numFmt numFmtId="164" formatCode="#,##0.000"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -461,7 +460,7 @@
         <v>Documented PERIOD_SCOPE_MISMATCH in UI metadata and certification report</v>
       </c>
       <c r="J2" t="str">
-        <v>2026-09-30T12:43:01.664Z</v>
+        <v>2026-09-30T17:56:52.911Z</v>
       </c>
     </row>
     <row r="3">
@@ -493,7 +492,7 @@
         <v>Unified regex to accept both alphanumeric and numeric SKUs; sample SKU aligned with unique items count</v>
       </c>
       <c r="J3" t="str">
-        <v>2026-09-30T12:43:01.664Z</v>
+        <v>2026-09-30T17:56:52.911Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>